<commit_message>
Refactor data handling by replacing DataTableInstance with ScenarioContext and remove unused dependencies
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginTestData.xlsx
+++ b/src/test/resources/testdata/LoginTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vijay\eclipse-workspace\Amazon2\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{032FEEEE-D2A0-4F48-B9AB-5CB5CC1FEE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56D4E5F5-DDF5-4661-B0E0-40DEDC49BEE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ValidLogin" sheetId="1" r:id="rId1"/>
@@ -113,9 +113,6 @@
     <t>TC005</t>
   </si>
   <si>
-    <t>Login using database credentials</t>
-  </si>
-  <si>
     <t>dbuser@example.com</t>
   </si>
   <si>
@@ -135,6 +132,9 @@
   </si>
   <si>
     <t>Standard</t>
+  </si>
+  <si>
+    <t>Login with database credentials</t>
   </si>
 </sst>
 </file>
@@ -684,42 +684,42 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
       </c>
       <c r="E2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" t="s">
         <v>29</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>30</v>
-      </c>
-      <c r="G2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
         <v>9</v>
       </c>
       <c r="E3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
         <v>33</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>34</v>
-      </c>
-      <c r="G3" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>